<commit_message>
Add clarifying-question column for unmasked perechen items
For each of the 22 "Не маскируется" rows, add a column with a
concrete example and a question to the customer asking exactly what
should be masked (whole document vs. specific field, organizational
control vs. PII masking, whether a custom PIIType is needed). Rows
already covered ("Маскируется"/"Частично") are left blank (—).

recalc.py still times out in this sandbox on the Сводка sheet's
percentage formula (same known limitation noted in the prior commit);
counts unchanged (4/4/22 of 30), verified by hand.
</commit_message>
<xml_diff>
--- a/docs/analysis/pokrytie-maskirovaniya-perechen-d8.xlsx
+++ b/docs/analysis/pokrytie-maskirovaniya-perechen-d8.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,12 +51,23 @@
     </font>
     <font>
       <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="002B4C8C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="001E7A4C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00AAAAAA"/>
       <sz val="9"/>
     </font>
     <font>
@@ -99,7 +110,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -114,6 +125,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FBE7E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDF2FB"/>
       </patternFill>
     </fill>
     <fill>
@@ -153,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -164,40 +180,46 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -565,15 +587,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -583,10 +606,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1">
+    <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Источник требований: Приложение №2 к приказу Генерального директора АО «Инвестиционная компания Д8» от 18.05.2026 № 26-18/05-1. Нумерация пунктов — как в оригинальном документе (подпункты без сквозной нумерации в исходнике перечислены как отдельные строки одного пункта). Статус «Маскируется» — покрыто встроенным типом PIIType платформы. «Частично» — тип есть, но формулировка заказчика шире. «Не маскируется» — вне скоупа PII-маскировщика (организационная/финансовая/IT-информация, не именованная сущность).</t>
+          <t>Источник требований: Приложение №2 к приказу Генерального директора АО «Инвестиционная компания Д8» от 18.05.2026 № 26-18/05-1. Нумерация пунктов — как в оригинальном документе (подпункты без сквозной нумерации в исходнике перечислены как отдельные строки одного пункта). Статус «Маскируется» — покрыто встроенным типом PIIType платформы. «Частично» — тип есть, но формулировка заказчика шире. «Не маскируется» — вне скоупа PII-маскировщика (организационная/финансовая/IT-информация, не именованная сущность). Для строк со статусом «Не маскируется» в столбце G — вопрос к заказчику с примером, чтобы уточнить, что конкретно ожидается маскировать по этому пункту.</t>
         </is>
       </c>
     </row>
@@ -621,6 +644,11 @@
           <t>Комментарий</t>
         </is>
       </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Вопрос к заказчику (для уточнения объёма маскирования)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -653,6 +681,11 @@
           <t>Организационная информация, не PII-сущность</t>
         </is>
       </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Обслуживание по индивидуальному тарифному плану с персональным менеджером Ивановым И.И.». Что именно маскировать: описание условий схемы целиком (текст) или только упоминания сотрудников/клиентов в нём (уже покрывается ФИО)?</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -675,7 +708,7 @@
           <t>PERSON / FULL_NAME</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Маскируется</t>
         </is>
@@ -683,6 +716,11 @@
       <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Прямое совпадение со встроенным типом</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -707,7 +745,7 @@
           <t>PASSPORT</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>Частично</t>
         </is>
@@ -715,6 +753,11 @@
       <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Встроен только паспорт РФ; иные виды документов — нет</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -739,7 +782,7 @@
           <t>ADDRESS</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Маскируется</t>
         </is>
@@ -747,6 +790,11 @@
       <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Прямое совпадение со встроенным типом</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -771,7 +819,7 @@
           <t>PHONE</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Маскируется</t>
         </is>
@@ -779,6 +827,11 @@
       <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Прямое совпадение со встроенным типом</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -803,7 +856,7 @@
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Маскируется</t>
         </is>
@@ -811,6 +864,11 @@
       <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Прямое совпадение со встроенным типом</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -835,7 +893,7 @@
           <t>PERSON (частично)</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>Частично</t>
         </is>
@@ -843,6 +901,11 @@
       <c r="F11" s="5" t="inlineStr">
         <is>
           <t>ФИО таких лиц распознаётся, но сама роль/связь («выгодоприобретатель», «бенефициар») — не отдельная сущность</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -867,7 +930,7 @@
           <t>PERSON / ORG (частично)</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>Частично</t>
         </is>
@@ -875,6 +938,11 @@
       <c r="F12" s="5" t="inlineStr">
         <is>
           <t>ФИО/наименование — да; внутренний уникальный код клиента — нет типа</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -909,6 +977,11 @@
           <t>Известный пробел: «Номер договора» не входит во встроенные типы, нужен кастомный тип</t>
         </is>
       </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Договор № ИС-2024/0817 от 12.03.2024». Нужен ли отдельный кастомный тип «НОМЕР_ДОГОВОРА» для номера и даты, или достаточно маскирования ФИО/сумм, упомянутых рядом в тексте?</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -941,6 +1014,11 @@
           <t>Номер счёта отдельно распознаётся (BANK_ACCOUNT), но содержание сделки — нет</t>
         </is>
       </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «По счёту № 40817810900000012345 клиента Иванова И.И. 15.03.2024 совершена сделка на покупку 100 акций Сбербанк на сумму 25 000 руб.». Номер счёта и ФИО уже маскируются — нужно ли дополнительно маскировать содержание сделки (актив, объём, сумму) как отдельную категорию?</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -973,6 +1051,11 @@
           <t>Финансово-операционные данные, не именованная сущность</t>
         </is>
       </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Клиенту Петрову П.П. предоставлен маржинальный заём в размере 500 000 руб. под 12% годовых». Маскировать ли сумму и условия займа отдельно от ФИО клиента (которое уже маскируется)?</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1005,6 +1088,11 @@
           <t>Финансово-операционные данные, не именованная сущность</t>
         </is>
       </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Задолженность клиента Сидорова С.С. по состоянию на 01.04.2024 составляет 150 000 руб.». Требуется ли маскировать сумму задолженности как отдельную категорию, или достаточно маскирования ФИО?</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1037,6 +1125,11 @@
           <t>Финансово-операционные данные, не именованная сущность</t>
         </is>
       </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Обязательство по сделке № 145 от 10.01.2024 признано прекращённым 20.02.2024 в связи с неисполнением». Что здесь требует маскирования: номер сделки, сам факт прекращения, обе части?</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1069,6 +1162,11 @@
           <t>Финансово-операционные данные, не именованная сущность</t>
         </is>
       </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Исходящий остаток по счёту клиента: 500 акций Газпром, плановый остаток на конец периода — 480 акций». Считаются ли такие цифры конфиденциальными сами по себе (без ФИО в той же фразе), и если да — нужен отдельный тип?</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1101,6 +1199,11 @@
           <t>Документ целиком; вложенные ФИО/суммы распознаются отдельно, но не как категория</t>
         </is>
       </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Поручение клиента Кузнецова К.К. на покупку 200 облигаций ОФЗ-26238 на сумму 210 000 руб.». Маскировать ли поручение как документ целиком, или только вложенные ФИО/суммы (уже покрыты существующими типами)?</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1133,6 +1236,11 @@
           <t>Аналогично п. 1.4</t>
         </is>
       </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Поручение на продажу 10 000 USD по курсу 92,50». Аналогично п. 1.4: маскировать текст поручения целиком или только сумму/курс как отдельную категорию?</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1155,7 +1263,7 @@
           <t>ORG (частично)</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>Частично</t>
         </is>
@@ -1163,6 +1271,11 @@
       <c r="F21" s="5" t="inlineStr">
         <is>
           <t>Название юрлица распознаётся, но сама информация о взаимоотношениях — нет</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1197,6 +1310,11 @@
           <t>Договорная информация, не PII-сущность</t>
         </is>
       </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «По агентскому соглашению с ООО «Брокер-Партнёр» комиссия составляет 0,15% от объёма сделок клиентов, привлечённых партнёром». Считаются ли условия соглашения (ставка, объём) данными для маскирования, или это регулируется NDA/договором вне PII-маскировщика?</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1229,6 +1347,11 @@
           <t>IT-инфраструктура, вне скоупа PII-маскировщика</t>
         </is>
       </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Доступ к модулю «Клиентские счета» имеют роли: Операционист, Старший операционист, Руководитель отдела». Подтвердите: этот пункт закрывается организационными/техническими мерами (RBAC, журналирование доступа), а не PII-маскировщиком?</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1261,6 +1384,11 @@
           <t>IT-инфраструктура, вне скоупа PII-маскировщика</t>
         </is>
       </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Сотруднику Смирнову А.А. предоставлен доступ уровня «Администратор» к CRM». ФИО сотрудника уже маскируется — нужно ли отдельно маскировать сам факт/уровень предоставленных прав доступа?</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1293,6 +1421,11 @@
           <t>IT-инфраструктура, вне скоупа PII-маскировщика</t>
         </is>
       </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Схема сети: DMZ 10.10.1.0/24 → firewall → внутренний сегмент 10.10.2.0/24, сервер itq-db-01». Нужен ли отдельный тип для IP-адресов/имён серверов (сейчас не входит во встроенные типы)?</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1325,6 +1458,11 @@
           <t>Исходный код, вне скоупа PII-маскировщика</t>
         </is>
       </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Пример: фрагмент внутреннего скрипта расчёта комиссии, вставленный в чат с ИИ. Требуется построчное маскирование кода, или предполагается полный запрет на передачу кода в ИИ (политика уровня п. 5.1) без частичного маскирования?</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1357,6 +1495,11 @@
           <t>Организационно-техническая ИБ-информация</t>
         </is>
       </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Используется двухфакторная аутентификация и шифрование AES-256 для хранения данных клиентов». Считать ли названия методов/технологий защиты данными для маскирования, или контроль обеспечивается запретом передачи таких документов в ИИ?</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1389,6 +1532,11 @@
           <t>Организационно-техническая ИБ-информация</t>
         </is>
       </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Сотрудники проходят проверку службой безопасности и подписывают NDA сроком на 3 года». Маскировать ли описание процедур, или только ФИО упомянутых сотрудников (уже покрывается)?</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1421,6 +1569,11 @@
           <t>Организационно-техническая ИБ-информация</t>
         </is>
       </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Резервный дата-центр расположен по адресу [адрес], время переключения — 15 минут». Маскировать ли адрес объекта (тип ADDRESS настроен на адреса физлиц, не гарантированно сработает на адрес ЦОД) и технические параметры?</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1453,6 +1606,11 @@
           <t>Организационно-техническая ИБ-информация</t>
         </is>
       </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Установлена система видеонаблюдения Hikvision DS-2CD2, СКУД Perco». Нужно ли маскировать названия/модели используемых средств защиты как отдельную категорию?</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1485,6 +1643,11 @@
           <t>Организационно-техническая ИБ-информация</t>
         </is>
       </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «Пропускной режим: турникеты на 1 этаже, пост охраны круглосуточно, видеонаблюдение периметра». Считается ли такое описание конфиденциальным для маскирования в документах, обрабатываемых ИИ?</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1517,6 +1680,11 @@
           <t>Организационно-техническая ИБ-информация</t>
         </is>
       </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>Пример: «По итогам пентеста в марте 2024 выявлено 3 уязвимости критического уровня в модуле авторизации». Маскировать ли содержание отчёта (находки, уязвимости) как отдельную категорию, или предполагается полный запрет на загрузку таких отчётов в систему?</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -1549,6 +1717,11 @@
           <t>Зонтичная политика («не отправлять в ИИ сведения из разделов 1–4»), не отдельный тип данных</t>
         </is>
       </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Пример: сотрудник загружает в чат с ИИ выписку по счёту клиента для анализа. Как должна работать проверка: блокировка загрузки документа целиком при обнаружении данных из разделов 1–4, или маскирование конкретных полей перед отправкой в модель?</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -1581,11 +1754,16 @@
           <t>Зонтичная политика, не отдельный тип данных</t>
         </is>
       </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Пример: ИИ в ответе процитировал фрагмент загруженного договора с ФИО и суммой. Должен ли ответ агента дополнительно проверяться/маскироваться перед показом пользователю, аналогично входящим документам?</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1606,85 +1784,85 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>СВОДКА ПО СТАТУСАМ</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Количество пунктов</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
         <is>
           <t>Доля</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Маскируется</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
+      <c r="B4" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C4" s="13">
+      <c r="C4" s="15">
         <f>B4/30</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Частично</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="15">
         <f>B5/30</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>Не маскируется</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="n">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Не маскируется</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="n">
         <v>22</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="15">
         <f>B6/30</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>Итого пунктов</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="18" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="9" ht="50" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>Пункты «Не маскируется» — это преимущественно разделы 2–5 Перечня (контрагенты, IT-инфраструктура, ИБ-меры, политика работы с ИИ) и часть раздела 1 (номера договоров, финансово-операционные детали) — они не являются именованными PII-сущностями и требуют либо кастомных типов, либо контроля на уровне разграничения доступа/DLP, а не PII-маскирования.</t>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Пункты «Не маскируется» — это преимущественно разделы 2–5 Перечня (контрагенты, IT-инфраструктура, ИБ-меры, политика работы с ИИ) и часть раздела 1 (номера договоров, финансово-операционные детали) — они не являются именованными PII-сущностями и требуют либо кастомных типов, либо контроля на уровне разграничения доступа/DLP, а не PII-маскирования. По каждому такому пункту в столбце «Вопрос к заказчику» на листе «Покрытие маскирования» сформулирован уточняющий вопрос с примером — ответы заказчика нужны, чтобы решить, где достаточно организационных/DLP-мер, а где требуется разработка кастомного PIIType.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add clarification-flag and reference-file columns to masking coverage
Two new columns in docs/analysis/pokrytie-maskirovaniya-perechen-d8.xlsx:
- F "Требуется уточнение, что именно маскировать" — Да/Нет flag,
  Да wherever a clarifying question already exists (all 22
  "Не маскируется" rows), for quick filtering.
- I "Название эталонных файлов для проверки маскирования" — maps
  each item to matching files in
  docs/test-data/anonymizer-2-test-documents/ (per manifest.json
  ground truth) that can be used to test that item's masking, or "—"
  when no existing test file covers it (mostly the financial/IT/InfoSec
  gaps, which were never modeled in the test-document set).
</commit_message>
<xml_diff>
--- a/docs/analysis/pokrytie-maskirovaniya-perechen-d8.xlsx
+++ b/docs/analysis/pokrytie-maskirovaniya-perechen-d8.xlsx
@@ -57,17 +57,17 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00AAAAAA"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="001E7A4C"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00AAAAAA"/>
       <sz val="9"/>
     </font>
     <font>
@@ -169,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -180,10 +180,10 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -192,10 +192,16 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -587,16 +593,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -606,10 +614,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
+    <row r="2" ht="76" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Источник требований: Приложение №2 к приказу Генерального директора АО «Инвестиционная компания Д8» от 18.05.2026 № 26-18/05-1. Нумерация пунктов — как в оригинальном документе (подпункты без сквозной нумерации в исходнике перечислены как отдельные строки одного пункта). Статус «Маскируется» — покрыто встроенным типом PIIType платформы. «Частично» — тип есть, но формулировка заказчика шире. «Не маскируется» — вне скоупа PII-маскировщика (организационная/финансовая/IT-информация, не именованная сущность). Для строк со статусом «Не маскируется» в столбце G — вопрос к заказчику с примером, чтобы уточнить, что конкретно ожидается маскировать по этому пункту.</t>
+          <t>Источник требований: Приложение №2 к приказу Генерального директора АО «Инвестиционная компания Д8» от 18.05.2026 № 26-18/05-1. Нумерация пунктов — как в оригинальном документе (подпункты без сквозной нумерации в исходнике перечислены как отдельные строки одного пункта). Статус «Маскируется» — покрыто встроенным типом PIIType платформы. «Частично» — тип есть, но формулировка заказчика шире. «Не маскируется» — вне скоупа PII-маскировщика (организационная/финансовая/IT-информация, не именованная сущность). Столбец F — краткий флаг: нужно ли уточнение объёма у заказчика (Да — для всех «Не маскируется», где полностью неясно, что относится к пункту). Столбец H — сам вопрос с примером. Столбец I — какие из уже готовых тестовых документов (docs/test-data/anonymizer-2-test-documents/, ground truth в manifest.json) можно использовать, чтобы прогнать и проверить маскирование по этому пункту; «—» значит, что подходящего документа в наборе пока нет и потребуется отдельный тестовый файл.</t>
         </is>
       </c>
     </row>
@@ -641,12 +649,22 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
+          <t>Требуется уточнение, что именно маскировать</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
           <t>Комментарий</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Вопрос к заказчику (для уточнения объёма маскирования)</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Название эталонных файлов для проверки маскирования</t>
         </is>
       </c>
     </row>
@@ -676,14 +694,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Организационная информация, не PII-сущность</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Пример: «Обслуживание по индивидуальному тарифному плану с персональным менеджером Ивановым И.И.». Что именно маскировать: описание условий схемы целиком (текст) или только упоминания сотрудников/клиентов в нём (уже покрывается ФИО)?</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>— (нет соответствующей сущности в текущем наборе)</t>
         </is>
       </c>
     </row>
@@ -708,19 +736,29 @@
           <t>PERSON / FULL_NAME</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Маскируется</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Прямое совпадение со встроенным типом</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>01-anketa-klienta, 02-sluzhebnaya-zapiska, 03-reestr-operaciy (все форматы; см. manifest.json, тип «ФИО»)</t>
         </is>
       </c>
     </row>
@@ -745,19 +783,29 @@
           <t>PASSPORT</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Частично</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Встроен только паспорт РФ; иные виды документов — нет</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>01-anketa-klienta (поля «Паспорт (серия+номер)», «Место выдачи паспорта»)</t>
         </is>
       </c>
     </row>
@@ -782,19 +830,29 @@
           <t>ADDRESS</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>Маскируется</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Прямое совпадение со встроенным типом</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>01-anketa-klienta, 02-sluzhebnaya-zapiska (тип «Адрес»)</t>
         </is>
       </c>
     </row>
@@ -819,19 +877,29 @@
           <t>PHONE</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>Маскируется</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Прямое совпадение со встроенным типом</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>01-anketa-klienta, 02-sluzhebnaya-zapiska, 03-reestr-operaciy (тип «Телефон»)</t>
         </is>
       </c>
     </row>
@@ -856,19 +924,29 @@
           <t>EMAIL</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>Маскируется</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Прямое совпадение со встроенным типом</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>01-anketa-klienta, 02-sluzhebnaya-zapiska (тип «Email»)</t>
         </is>
       </c>
     </row>
@@ -893,19 +971,29 @@
           <t>PERSON (частично)</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Частично</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>ФИО таких лиц распознаётся, но сама роль/связь («выгодоприобретатель», «бенефициар») — не отдельная сущность</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>— (роль/связь как отдельная сущность в наборе не смоделирована; ФИО — см. п. 1.2 выше)</t>
         </is>
       </c>
     </row>
@@ -930,19 +1018,29 @@
           <t>PERSON / ORG (частично)</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>Частично</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>ФИО/наименование — да; внутренний уникальный код клиента — нет типа</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>01-anketa-klienta, 02-sluzhebnaya-zapiska, 03-reestr-operaciy (только ФИО; уникальный код клиента в наборе не смоделирован)</t>
         </is>
       </c>
     </row>
@@ -972,14 +1070,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>Известный пробел: «Номер договора» не входит во встроенные типы, нужен кастомный тип</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>Пример: «Договор № ИС-2024/0817 от 12.03.2024». Нужен ли отдельный кастомный тип «НОМЕР_ДОГОВОРА» для номера и даты, или достаточно маскирования ФИО/сумм, упомянутых рядом в тексте?</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>01-anketa-klienta, 02-sluzhebnaya-zapiska, 03-reestr-operaciy (поле «Номер договора»; отдельная «дата договора» в наборе не смоделирована)</t>
         </is>
       </c>
     </row>
@@ -1009,14 +1117,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>Номер счёта отдельно распознаётся (BANK_ACCOUNT), но содержание сделки — нет</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>Пример: «По счёту № 40817810900000012345 клиента Иванова И.И. 15.03.2024 совершена сделка на покупку 100 акций Сбербанк на сумму 25 000 руб.». Номер счёта и ФИО уже маскируются — нужно ли дополнительно маскировать содержание сделки (актив, объём, сумму) как отдельную категорию?</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>02-sluzhebnaya-zapiska (поля «Сумма операции», «Дата операции»), 03-reestr-operaciy (реестр из 5 операций)</t>
         </is>
       </c>
     </row>
@@ -1046,14 +1164,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>Финансово-операционные данные, не именованная сущность</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>Пример: «Клиенту Петрову П.П. предоставлен маржинальный заём в размере 500 000 руб. под 12% годовых». Маскировать ли сумму и условия займа отдельно от ФИО клиента (которое уже маскируется)?</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>— (нет соответствующей сущности в текущем наборе, нужен отдельный документ)</t>
         </is>
       </c>
     </row>
@@ -1083,14 +1211,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>Финансово-операционные данные, не именованная сущность</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>Пример: «Задолженность клиента Сидорова С.С. по состоянию на 01.04.2024 составляет 150 000 руб.». Требуется ли маскировать сумму задолженности как отдельную категорию, или достаточно маскирования ФИО?</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>— (нет соответствующей сущности в текущем наборе, нужен отдельный документ)</t>
         </is>
       </c>
     </row>
@@ -1120,14 +1258,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>Финансово-операционные данные, не именованная сущность</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>Пример: «Обязательство по сделке № 145 от 10.01.2024 признано прекращённым 20.02.2024 в связи с неисполнением». Что здесь требует маскирования: номер сделки, сам факт прекращения, обе части?</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>— (нет соответствующей сущности в текущем наборе, нужен отдельный документ)</t>
         </is>
       </c>
     </row>
@@ -1157,14 +1305,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>Финансово-операционные данные, не именованная сущность</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>Пример: «Исходящий остаток по счёту клиента: 500 акций Газпром, плановый остаток на конец периода — 480 акций». Считаются ли такие цифры конфиденциальными сами по себе (без ФИО в той же фразе), и если да — нужен отдельный тип?</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>— (нет соответствующей сущности в текущем наборе, нужен отдельный документ)</t>
         </is>
       </c>
     </row>
@@ -1194,14 +1352,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>Документ целиком; вложенные ФИО/суммы распознаются отдельно, но не как категория</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>Пример: «Поручение клиента Кузнецова К.К. на покупку 200 облигаций ОФЗ-26238 на сумму 210 000 руб.». Маскировать ли поручение как документ целиком, или только вложенные ФИО/суммы (уже покрыты существующими типами)?</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>— (в наборе нет документа-поручения; ближайший по смыслу — 03-reestr-operaciy, но это не поручение)</t>
         </is>
       </c>
     </row>
@@ -1231,14 +1399,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>Аналогично п. 1.4</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>Пример: «Поручение на продажу 10 000 USD по курсу 92,50». Аналогично п. 1.4: маскировать текст поручения целиком или только сумму/курс как отдельную категорию?</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>— (нет соответствующей сущности в текущем наборе, нужен отдельный документ)</t>
         </is>
       </c>
     </row>
@@ -1263,19 +1441,29 @@
           <t>ORG (частично)</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Частично</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>Название юрлица распознаётся, но сама информация о взаимоотношениях — нет</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="H21" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>— (в наборе нет документа с юрлицами-контрагентами)</t>
         </is>
       </c>
     </row>
@@ -1305,14 +1493,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>Договорная информация, не PII-сущность</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="H22" s="7" t="inlineStr">
         <is>
           <t>Пример: «По агентскому соглашению с ООО «Брокер-Партнёр» комиссия составляет 0,15% от объёма сделок клиентов, привлечённых партнёром». Считаются ли условия соглашения (ставка, объём) данными для маскирования, или это регулируется NDA/договором вне PII-маскировщика?</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>— (нет соответствующей сущности в текущем наборе, нужен отдельный документ)</t>
         </is>
       </c>
     </row>
@@ -1342,14 +1540,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>IT-инфраструктура, вне скоупа PII-маскировщика</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>Пример: «Доступ к модулю «Клиентские счета» имеют роли: Операционист, Старший операционист, Руководитель отдела». Подтвердите: этот пункт закрывается организационными/техническими мерами (RBAC, журналирование доступа), а не PII-маскировщиком?</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>— (не PII-документ, вне охвата test-tracker)</t>
         </is>
       </c>
     </row>
@@ -1379,14 +1587,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>IT-инфраструктура, вне скоупа PII-маскировщика</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="H24" s="7" t="inlineStr">
         <is>
           <t>Пример: «Сотруднику Смирнову А.А. предоставлен доступ уровня «Администратор» к CRM». ФИО сотрудника уже маскируется — нужно ли отдельно маскировать сам факт/уровень предоставленных прав доступа?</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>— (не PII-документ, вне охвата test-tracker)</t>
         </is>
       </c>
     </row>
@@ -1416,14 +1634,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>IT-инфраструктура, вне скоупа PII-маскировщика</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="H25" s="7" t="inlineStr">
         <is>
           <t>Пример: «Схема сети: DMZ 10.10.1.0/24 → firewall → внутренний сегмент 10.10.2.0/24, сервер itq-db-01». Нужен ли отдельный тип для IP-адресов/имён серверов (сейчас не входит во встроенные типы)?</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>— (не PII-документ, вне охвата test-tracker)</t>
         </is>
       </c>
     </row>
@@ -1453,14 +1681,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>Исходный код, вне скоупа PII-маскировщика</t>
         </is>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="H26" s="7" t="inlineStr">
         <is>
           <t>Пример: фрагмент внутреннего скрипта расчёта комиссии, вставленный в чат с ИИ. Требуется построчное маскирование кода, или предполагается полный запрет на передачу кода в ИИ (политика уровня п. 5.1) без частичного маскирования?</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>— (не PII-документ, вне охвата test-tracker)</t>
         </is>
       </c>
     </row>
@@ -1490,14 +1728,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
         <is>
           <t>Организационно-техническая ИБ-информация</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="H27" s="7" t="inlineStr">
         <is>
           <t>Пример: «Используется двухфакторная аутентификация и шифрование AES-256 для хранения данных клиентов». Считать ли названия методов/технологий защиты данными для маскирования, или контроль обеспечивается запретом передачи таких документов в ИИ?</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>— (не PII-документ, вне охвата test-tracker)</t>
         </is>
       </c>
     </row>
@@ -1527,14 +1775,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>Организационно-техническая ИБ-информация</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="H28" s="7" t="inlineStr">
         <is>
           <t>Пример: «Сотрудники проходят проверку службой безопасности и подписывают NDA сроком на 3 года». Маскировать ли описание процедур, или только ФИО упомянутых сотрудников (уже покрывается)?</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>— (не PII-документ, вне охвата test-tracker)</t>
         </is>
       </c>
     </row>
@@ -1564,14 +1822,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
         <is>
           <t>Организационно-техническая ИБ-информация</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="H29" s="7" t="inlineStr">
         <is>
           <t>Пример: «Резервный дата-центр расположен по адресу [адрес], время переключения — 15 минут». Маскировать ли адрес объекта (тип ADDRESS настроен на адреса физлиц, не гарантированно сработает на адрес ЦОД) и технические параметры?</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>— (не PII-документ, вне охвата test-tracker)</t>
         </is>
       </c>
     </row>
@@ -1601,14 +1869,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>Организационно-техническая ИБ-информация</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="H30" s="7" t="inlineStr">
         <is>
           <t>Пример: «Установлена система видеонаблюдения Hikvision DS-2CD2, СКУД Perco». Нужно ли маскировать названия/модели используемых средств защиты как отдельную категорию?</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>— (не PII-документ, вне охвата test-tracker)</t>
         </is>
       </c>
     </row>
@@ -1638,14 +1916,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>Организационно-техническая ИБ-информация</t>
         </is>
       </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="H31" s="7" t="inlineStr">
         <is>
           <t>Пример: «Пропускной режим: турникеты на 1 этаже, пост охраны круглосуточно, видеонаблюдение периметра». Считается ли такое описание конфиденциальным для маскирования в документах, обрабатываемых ИИ?</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>— (не PII-документ, вне охвата test-tracker)</t>
         </is>
       </c>
     </row>
@@ -1675,14 +1963,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>Организационно-техническая ИБ-информация</t>
         </is>
       </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="H32" s="7" t="inlineStr">
         <is>
           <t>Пример: «По итогам пентеста в марте 2024 выявлено 3 уязвимости критического уровня в модуле авторизации». Маскировать ли содержание отчёта (находки, уязвимости) как отдельную категорию, или предполагается полный запрет на загрузку таких отчётов в систему?</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>— (не PII-документ, вне охвата test-tracker)</t>
         </is>
       </c>
     </row>
@@ -1712,14 +2010,24 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>Зонтичная политика («не отправлять в ИИ сведения из разделов 1–4»), не отдельный тип данных</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="H33" s="7" t="inlineStr">
         <is>
           <t>Пример: сотрудник загружает в чат с ИИ выписку по счёту клиента для анализа. Как должна работать проверка: блокировка загрузки документа целиком при обнаружении данных из разделов 1–4, или маскирование конкретных полей перед отправкой в модель?</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>— (политика уровня загрузки, не конкретный документ; для прогона см. любой файл из test-tracker.xlsx)</t>
         </is>
       </c>
     </row>
@@ -1749,21 +2057,31 @@
           <t>Не маскируется</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>Зонтичная политика, не отдельный тип данных</t>
         </is>
       </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="H34" s="7" t="inlineStr">
         <is>
           <t>Пример: ИИ в ответе процитировал фрагмент загруженного договора с ФИО и суммой. Должен ли ответ агента дополнительно проверяться/маскироваться перед показом пользователю, аналогично входящим документам?</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>— (политика уровня ответа агента, не конкретный документ)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1784,83 +2102,83 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>СВОДКА ПО СТАТУСАМ</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>Количество пунктов</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>Доля</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>Маскируется</t>
         </is>
       </c>
-      <c r="B4" s="14" t="n">
+      <c r="B4" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="17">
         <f>B4/30</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>Частично</t>
         </is>
       </c>
-      <c r="B5" s="14" t="n">
+      <c r="B5" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="17">
         <f>B5/30</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>Не маскируется</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="n">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>Не маскируется</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
         <v>22</v>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="17">
         <f>B6/30</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>Итого пунктов</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="20" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Пункты «Не маскируется» — это преимущественно разделы 2–5 Перечня (контрагенты, IT-инфраструктура, ИБ-меры, политика работы с ИИ) и часть раздела 1 (номера договоров, финансово-операционные детали) — они не являются именованными PII-сущностями и требуют либо кастомных типов, либо контроля на уровне разграничения доступа/DLP, а не PII-маскирования. По каждому такому пункту в столбце «Вопрос к заказчику» на листе «Покрытие маскирования» сформулирован уточняющий вопрос с примером — ответы заказчика нужны, чтобы решить, где достаточно организационных/DLP-мер, а где требуется разработка кастомного PIIType.</t>
         </is>

</xml_diff>

<commit_message>
Add CustomPIIType config proposals for unclosed masking types
New section on the "Три слоя маскирования" sheet, based on the vendor's
PII-Shield span-registry doc: concrete id/prefix/regex/validator configs
for contract number, client code, and internal hostname — the three
items in Layer 1 not covered by built-in PIIType.
</commit_message>
<xml_diff>
--- a/docs/analysis/pokrytie-maskirovaniya-perechen-d8.xlsx
+++ b/docs/analysis/pokrytie-maskirovaniya-perechen-d8.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -170,6 +170,12 @@
       <color rgb="00A8393B"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="005A3E85"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -235,7 +241,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -337,6 +343,7 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2369,7 +2376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3748,13 +3755,205 @@
         </is>
       </c>
     </row>
+    <row r="58" ht="24" customHeight="1">
+      <c r="A58" s="43" t="inlineStr">
+        <is>
+          <t>РАЗДЕЛ 4 — Предлагаемые конфиги CustomPIIType для незакрытых пунктов (п. 1.3, 3.3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="76" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Источник механизма: docs/sources/pii-shield-masking-span-registry.docx, §2 «Кастомные типы (CustomPIIType)» — новый тип маскирования добавляется БЕЗ изменения кода платформы, через конфиг / Admin API (pii_shield/config.py:151-200), полями id (slug), prefix (UPPERCASE → токен [PREFIX_N]), display_name, patterns (regex + флаги + min_confidence + опциональный валидатор), enabled. Количество типов не ограничено. Ниже — конкретные предложения по трём типам из Слоя 1 (см. таблицу выше), которые сегодня не входят во встроенные PIIType. Regex взяты из таблицы Слоя 1 этого листа; для всех трёх контрольной суммы нет (валидатор не нужен), поле «Валидатор» оставлено пустым намеренно. min_confidence — предлагаемые стартовые значения, требуют калибровки на реальных документах Д8 в ходе пилота.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="29" t="inlineStr">
+        <is>
+          <t>Пункт Перечня</t>
+        </is>
+      </c>
+      <c r="B60" s="29" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C60" s="29" t="inlineStr">
+        <is>
+          <t>prefix → токен маски</t>
+        </is>
+      </c>
+      <c r="D60" s="29" t="inlineStr">
+        <is>
+          <t>display_name</t>
+        </is>
+      </c>
+      <c r="E60" s="29" t="inlineStr">
+        <is>
+          <t>Regex-паттерн (patterns)</t>
+        </is>
+      </c>
+      <c r="F60" s="29" t="inlineStr">
+        <is>
+          <t>Валидатор</t>
+        </is>
+      </c>
+      <c r="G60" s="29" t="inlineStr">
+        <is>
+          <t>min_confidence (предложение)</t>
+        </is>
+      </c>
+      <c r="H60" s="29" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>contract_num</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>CONTRACT → [CONTRACT_N]</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Номер договора Д8</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>№?\s?[А-ЯA-Z]{2,10}(?:[\-/][A-Za-zА-я0-9]+){1,5}</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>Открытый вопрос заказчику: подтвердить формат номеров договоров по всем подразделениям — regex построен по единственному примеру из Перечня (ИКД-1-PRO-TEST-001), реальная вариативность формата не подтверждена</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>client_code</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>CL → [CL_N]</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Уникальный код клиента</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>CL[\-_]?\d{4,8}</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>Открытый вопрос заказчику: формат гипотетический (CL-000482), реальный шаблон кода клиента у заказчика не подтверждён</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>internal_hostname</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>HOSTNAME → [HOSTNAME_N]</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Внутренний хостнейм</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>[a-z0-9]([a-z0-9\-]{0,61}[a-z0-9])?\.(?:local|internal|corp)\b</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>Открытый вопрос заказчику: подтвердить домен(ы) внутренней сети — .local/.internal/.corp здесь заглушка; более узкий min_confidence из-за риска ловить произвольные слова с точкой</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="32" customHeight="1">
+      <c r="A65" s="26" t="inlineStr">
+        <is>
+          <t>Все три — «Низкая» надёжность в Слое 1 выше именно по этой причине: включение в enabled=true до подтверждения формата заказчиком создаёт риск ложных срабатываний. Рекомендация: включать по одному, с проверкой на реальных документах пилота, а не все три сразу.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="12">
     <mergeCell ref="A29:I29"/>
+    <mergeCell ref="A59:I59"/>
+    <mergeCell ref="A65:I65"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A56:I56"/>
     <mergeCell ref="A30:I30"/>
+    <mergeCell ref="A58:I58"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A20:I20"/>
     <mergeCell ref="A21:I21"/>
@@ -4244,11 +4443,6 @@
           <t>ГЛАВНОЕ РЕШЕНИЕ: МАРШРУТИЗАЦИЯ ПО КАНАЛУ, А НЕ ЕДИНАЯ НАСТРОЙКА МАСКИРОВАНИЯ</t>
         </is>
       </c>
-      <c r="B4" s="33" t="n"/>
-      <c r="C4" s="33" t="n"/>
-      <c r="D4" s="33" t="n"/>
-      <c r="E4" s="33" t="n"/>
-      <c r="F4" s="33" t="n"/>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="34" t="inlineStr">
@@ -4314,11 +4508,6 @@
           <t>РАСШИРЕННЫЙ СПИСОК МАСКИРУЕМЫХ ПОЛЕЙ — ДЛЯ КАНАЛА Б (ВНЕШНЯЯ МОДЕЛЬ)</t>
         </is>
       </c>
-      <c r="B10" s="33" t="n"/>
-      <c r="C10" s="33" t="n"/>
-      <c r="D10" s="33" t="n"/>
-      <c r="E10" s="33" t="n"/>
-      <c r="F10" s="33" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
@@ -4524,11 +4713,6 @@
           <t>ПОРТФЕЛЬ И ОСТАТКИ — ЕДИНСТВЕННОЕ ПОЛЕ БЕЗ ЧИСТОГО РЕШЕНИЯ В КАНАЛЕ Б</t>
         </is>
       </c>
-      <c r="B21" s="42" t="n"/>
-      <c r="C21" s="42" t="n"/>
-      <c r="D21" s="42" t="n"/>
-      <c r="E21" s="42" t="n"/>
-      <c r="F21" s="42" t="n"/>
     </row>
     <row r="22" ht="58" customHeight="1">
       <c r="A22" s="34" t="inlineStr">
@@ -4611,11 +4795,6 @@
           <t>ДОКУМЕНТ-УРОВНЕВАЯ DLP-ПОЛИТИКА (ДЛЯ КАНАЛА Б)</t>
         </is>
       </c>
-      <c r="B28" s="33" t="n"/>
-      <c r="C28" s="33" t="n"/>
-      <c r="D28" s="33" t="n"/>
-      <c r="E28" s="33" t="n"/>
-      <c r="F28" s="33" t="n"/>
     </row>
     <row r="29" ht="76" customHeight="1">
       <c r="A29" s="34" t="inlineStr">
@@ -4630,11 +4809,6 @@
           <t>ОСТАТОЧНЫЙ РИСК ПОСЛЕ ВСЕХ МЕР — ЧЕСТНО, БЕЗ ПРИУКРАШИВАНИЯ</t>
         </is>
       </c>
-      <c r="B31" s="36" t="n"/>
-      <c r="C31" s="36" t="n"/>
-      <c r="D31" s="36" t="n"/>
-      <c r="E31" s="36" t="n"/>
-      <c r="F31" s="36" t="n"/>
     </row>
     <row r="32" ht="70" customHeight="1">
       <c r="A32" s="37" t="inlineStr">
@@ -4642,11 +4816,6 @@
           <t>Схема выше сводит риск к практически управляемому уровню, но не к нулю — «нет утечки» в абсолютном смысле недостижимо, если бизнесу всё же нужна точная работа с портфельными данными через внешнюю модель (вариант «обобщение чисел» или «контрактная мера» выше). Честная формулировка для заказчика: риск снижается с «прямая деанонимизация клиента по открытым данным» (текущее состояние) до «остаточный риск при инсайдерской угрозе или редком сценарии корреляции с внешней утечкой» (после внедрения схемы) — это управляемый, а не нулевой уровень. Единственный канал с формально нулевым риском выхода данных — канал А (внутренняя модель), и для класса документов вроде «Отчёт брокера» именно он должен быть путём по умолчанию.</t>
         </is>
       </c>
-      <c r="B32" s="36" t="n"/>
-      <c r="C32" s="36" t="n"/>
-      <c r="D32" s="36" t="n"/>
-      <c r="E32" s="36" t="n"/>
-      <c r="F32" s="36" t="n"/>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="32" t="inlineStr">
@@ -4654,11 +4823,6 @@
           <t>ЧЕК-ЛИСТ ВНЕДРЕНИЯ</t>
         </is>
       </c>
-      <c r="B34" s="33" t="n"/>
-      <c r="C34" s="33" t="n"/>
-      <c r="D34" s="33" t="n"/>
-      <c r="E34" s="33" t="n"/>
-      <c r="F34" s="33" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="29" t="inlineStr">

</xml_diff>